<commit_message>
chore: prepare lite converter deployment
</commit_message>
<xml_diff>
--- a/tests/fixtures/itinerary-golden/싱가폴 3박 24년 10월 15일-QA00570979001 ASP211241015OZC기준  8+0 (2).xlsx
+++ b/tests/fixtures/itinerary-golden/싱가폴 3박 24년 10월 15일-QA00570979001 ASP211241015OZC기준  8+0 (2).xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hana\OneDrive - hanatour.com\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yoon/Desktop/tour-editor/tests/fixtures/itinerary-golden/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA0CE146-737E-4AD1-AE7D-0978A7470CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FDDBD3-F490-E948-851D-7DD9E3503243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57490" yWindow="8010" windowWidth="29020" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13140" yWindow="4140" windowWidth="29020" windowHeight="28280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="세부내역서" sheetId="12" r:id="rId1"/>
-    <sheet name="일정표" sheetId="9" r:id="rId2"/>
+    <sheet name="일정표" sheetId="9" r:id="rId1"/>
+    <sheet name="세부내역서" sheetId="12" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -745,12 +745,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
+    <numFmt numFmtId="6" formatCode="&quot;₩&quot;#,##0_);[Red]\(&quot;₩&quot;#,##0\)"/>
     <numFmt numFmtId="26" formatCode="\$#,##0.00_);[Red]\(\$#,##0.00\)"/>
     <numFmt numFmtId="176" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
-    <numFmt numFmtId="177" formatCode="&quot;₩&quot;#,##0_);[Red]\(&quot;₩&quot;#,##0\)"/>
-    <numFmt numFmtId="178" formatCode="#,##0.00_);[Red]\(#,##0.00\)"/>
-    <numFmt numFmtId="179" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
+    <numFmt numFmtId="177" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -1639,13 +1638,13 @@
     <xf numFmtId="176" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="26" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1744,34 +1743,34 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="40" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="40" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="40" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1816,7 +1815,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="15" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1849,7 +1848,7 @@
     <xf numFmtId="20" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1876,6 +1875,138 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1885,19 +2016,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1915,308 +2034,188 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="31" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="31" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2263,8 +2262,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="114300" y="171450"/>
-          <a:ext cx="9023350" cy="405065"/>
+          <a:off x="110873" y="171450"/>
+          <a:ext cx="9021032" cy="416757"/>
           <a:chOff x="35475" y="223538"/>
           <a:chExt cx="9166698" cy="516096"/>
         </a:xfrm>
@@ -2747,1086 +2746,314 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17"/>
-  <cols>
-    <col min="1" max="1" width="9" style="32"/>
-    <col min="2" max="2" width="8.75" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.58203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="33" style="32" customWidth="1"/>
-    <col min="5" max="5" width="9.75" style="32" customWidth="1"/>
-    <col min="6" max="6" width="10" style="32" customWidth="1"/>
-    <col min="7" max="7" width="8.75" style="32" customWidth="1"/>
-    <col min="8" max="8" width="25.25" style="32" customWidth="1"/>
-    <col min="9" max="11" width="8.75" style="32" customWidth="1"/>
-    <col min="12" max="13" width="9" style="32"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" ht="16.5" customHeight="1" thickBot="1"/>
-    <row r="2" spans="1:13" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B2" s="118" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="119"/>
-      <c r="D2" s="84" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="120" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="121"/>
-      <c r="G2" s="121"/>
-      <c r="H2" s="122"/>
-    </row>
-    <row r="3" spans="1:13" ht="33.75" customHeight="1">
-      <c r="B3" s="123" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="124"/>
-      <c r="D3" s="57" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="125" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="127"/>
-    </row>
-    <row r="4" spans="1:13" ht="33.75" customHeight="1" thickBot="1">
-      <c r="B4" s="134" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="135"/>
-      <c r="D4" s="53" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="128"/>
-      <c r="F4" s="129"/>
-      <c r="G4" s="129"/>
-      <c r="H4" s="130"/>
-    </row>
-    <row r="5" spans="1:13" ht="33.75" customHeight="1">
-      <c r="B5" s="136" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="9">
-        <v>8</v>
-      </c>
-      <c r="E5" s="128"/>
-      <c r="F5" s="129"/>
-      <c r="G5" s="129"/>
-      <c r="H5" s="130"/>
-    </row>
-    <row r="6" spans="1:13" ht="22.5" customHeight="1">
-      <c r="B6" s="138" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="139"/>
-      <c r="D6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="128"/>
-      <c r="F6" s="129"/>
-      <c r="G6" s="129"/>
-      <c r="H6" s="130"/>
-    </row>
-    <row r="7" spans="1:13" ht="29.25" customHeight="1">
-      <c r="B7" s="138" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="139"/>
-      <c r="D7" s="56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="128"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="130"/>
-    </row>
-    <row r="8" spans="1:13" ht="27.75" customHeight="1">
-      <c r="B8" s="140" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="12">
-        <f>H37</f>
-        <v>983.5</v>
-      </c>
-      <c r="E8" s="128"/>
-      <c r="F8" s="129"/>
-      <c r="G8" s="129"/>
-      <c r="H8" s="130"/>
-    </row>
-    <row r="9" spans="1:13" ht="27" customHeight="1">
-      <c r="B9" s="141"/>
-      <c r="C9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="11">
-        <v>1000</v>
-      </c>
-      <c r="E9" s="128"/>
-      <c r="F9" s="129"/>
-      <c r="G9" s="129"/>
-      <c r="H9" s="130"/>
-    </row>
-    <row r="10" spans="1:13" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B10" s="142"/>
-      <c r="C10" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="13">
-        <f>D8*D9</f>
-        <v>983500</v>
-      </c>
-      <c r="E10" s="131"/>
-      <c r="F10" s="132"/>
-      <c r="G10" s="132"/>
-      <c r="H10" s="133"/>
-    </row>
-    <row r="11" spans="1:13" ht="38.25" customHeight="1" thickBot="1">
-      <c r="B11" s="109" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="109"/>
-      <c r="D11" s="82" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="114" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="115"/>
-      <c r="G11" s="115"/>
-      <c r="H11" s="115"/>
-    </row>
-    <row r="12" spans="1:13" ht="22.5" customHeight="1">
-      <c r="B12" s="110" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="112" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="112" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="112" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="112" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="112"/>
-      <c r="H12" s="116" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" s="3" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
-      <c r="A13" s="2"/>
-      <c r="B13" s="111"/>
-      <c r="C13" s="113"/>
-      <c r="D13" s="113"/>
-      <c r="E13" s="113"/>
-      <c r="F13" s="86" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="86" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" s="117"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" s="3" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="107" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="14">
-        <v>220</v>
-      </c>
-      <c r="F14" s="14">
-        <v>3</v>
-      </c>
-      <c r="G14" s="14">
-        <v>4</v>
-      </c>
-      <c r="H14" s="15">
-        <f>E14*F14*G14</f>
-        <v>2640</v>
-      </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" s="3" customFormat="1" ht="21" customHeight="1" thickBot="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="108"/>
-      <c r="C15" s="89"/>
-      <c r="D15" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="17">
-        <v>0</v>
-      </c>
-      <c r="F15" s="17">
-        <v>0</v>
-      </c>
-      <c r="G15" s="17">
-        <v>0</v>
-      </c>
-      <c r="H15" s="18">
-        <f>SUM(E15*F15*G15)</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" s="3" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="93" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="88" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="20">
-        <v>500</v>
-      </c>
-      <c r="F16" s="21">
-        <v>4</v>
-      </c>
-      <c r="G16" s="21">
-        <v>1</v>
-      </c>
-      <c r="H16" s="15">
-        <f t="shared" ref="H16:H26" si="0">E16*F16*G16</f>
-        <v>2000</v>
-      </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B17" s="94"/>
-      <c r="C17" s="83"/>
-      <c r="D17" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" s="35">
-        <v>60</v>
-      </c>
-      <c r="F17" s="36">
-        <v>1</v>
-      </c>
-      <c r="G17" s="36">
-        <v>1</v>
-      </c>
-      <c r="H17" s="33">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B18" s="94"/>
-      <c r="C18" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="24">
-        <v>0</v>
-      </c>
-      <c r="F18" s="37">
-        <v>0</v>
-      </c>
-      <c r="G18" s="37">
-        <v>0</v>
-      </c>
-      <c r="H18" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B19" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="85" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="46">
-        <v>1000</v>
-      </c>
-      <c r="F19" s="38">
-        <v>1</v>
-      </c>
-      <c r="G19" s="38">
-        <v>1</v>
-      </c>
-      <c r="H19" s="39">
-        <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B20" s="95"/>
-      <c r="C20" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="47">
-        <v>10</v>
-      </c>
-      <c r="F20" s="40">
-        <v>3</v>
-      </c>
-      <c r="G20" s="40">
-        <v>8</v>
-      </c>
-      <c r="H20" s="25">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B21" s="104" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="106" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="E21" s="48">
-        <v>20</v>
-      </c>
-      <c r="F21" s="36">
-        <v>1</v>
-      </c>
-      <c r="G21" s="36">
-        <v>8</v>
-      </c>
-      <c r="H21" s="39">
-        <f t="shared" si="0"/>
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B22" s="105"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E22" s="49">
-        <v>31</v>
-      </c>
-      <c r="F22" s="36">
-        <v>1</v>
-      </c>
-      <c r="G22" s="36">
-        <v>8</v>
-      </c>
-      <c r="H22" s="33">
-        <f t="shared" si="0"/>
-        <v>248</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B23" s="105"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="49">
-        <v>20</v>
-      </c>
-      <c r="F23" s="36">
-        <v>1</v>
-      </c>
-      <c r="G23" s="36">
-        <v>8</v>
-      </c>
-      <c r="H23" s="33">
-        <f t="shared" si="0"/>
-        <v>160</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B24" s="105"/>
-      <c r="C24" s="97"/>
-      <c r="D24" s="87"/>
-      <c r="E24" s="54">
-        <v>0</v>
-      </c>
-      <c r="F24" s="37">
-        <v>1</v>
-      </c>
-      <c r="G24" s="37">
-        <v>0</v>
-      </c>
-      <c r="H24" s="44">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" ht="22.5" customHeight="1">
-      <c r="B25" s="105"/>
-      <c r="C25" s="97"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="54">
-        <v>0</v>
-      </c>
-      <c r="F25" s="37">
-        <v>1</v>
-      </c>
-      <c r="G25" s="37">
-        <v>0</v>
-      </c>
-      <c r="H25" s="44">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B26" s="105"/>
-      <c r="C26" s="97"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="54">
-        <v>0</v>
-      </c>
-      <c r="F26" s="37">
-        <v>1</v>
-      </c>
-      <c r="G26" s="37">
-        <v>0</v>
-      </c>
-      <c r="H26" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B27" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="96" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="E27" s="55">
-        <v>20</v>
-      </c>
-      <c r="F27" s="38">
-        <v>1</v>
-      </c>
-      <c r="G27" s="38">
-        <v>8</v>
-      </c>
-      <c r="H27" s="39">
-        <f>E27*F27*G27</f>
-        <v>160</v>
-      </c>
-    </row>
-    <row r="28" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B28" s="93"/>
-      <c r="C28" s="97"/>
-      <c r="D28" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="E28" s="50">
-        <v>32</v>
-      </c>
-      <c r="F28" s="36">
-        <v>1</v>
-      </c>
-      <c r="G28" s="36">
-        <v>8</v>
-      </c>
-      <c r="H28" s="44">
-        <f t="shared" ref="H28:H35" si="1">E28*F28*G28</f>
-        <v>256</v>
-      </c>
-    </row>
-    <row r="29" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B29" s="93"/>
-      <c r="C29" s="97"/>
-      <c r="D29" s="43" t="s">
-        <v>48</v>
-      </c>
-      <c r="E29" s="50">
-        <v>18</v>
-      </c>
-      <c r="F29" s="36">
-        <v>1</v>
-      </c>
-      <c r="G29" s="36">
-        <v>8</v>
-      </c>
-      <c r="H29" s="44">
-        <f t="shared" si="1"/>
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B30" s="93"/>
-      <c r="C30" s="97"/>
-      <c r="D30" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="E30" s="50">
-        <v>20</v>
-      </c>
-      <c r="F30" s="36">
-        <v>1</v>
-      </c>
-      <c r="G30" s="36">
-        <v>8</v>
-      </c>
-      <c r="H30" s="44">
-        <f t="shared" si="1"/>
-        <v>160</v>
-      </c>
-    </row>
-    <row r="31" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B31" s="93"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="E31" s="50">
-        <v>55</v>
-      </c>
-      <c r="F31" s="36">
-        <v>1</v>
-      </c>
-      <c r="G31" s="36">
-        <v>8</v>
-      </c>
-      <c r="H31" s="44">
-        <f t="shared" si="1"/>
-        <v>440</v>
-      </c>
-    </row>
-    <row r="32" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B32" s="93"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="E32" s="50">
-        <v>25</v>
-      </c>
-      <c r="F32" s="36">
-        <v>1</v>
-      </c>
-      <c r="G32" s="36">
-        <v>8</v>
-      </c>
-      <c r="H32" s="44">
-        <f t="shared" si="1"/>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="33" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B33" s="93"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E33" s="50">
-        <v>0</v>
-      </c>
-      <c r="F33" s="36">
-        <v>1</v>
-      </c>
-      <c r="G33" s="36">
-        <v>0</v>
-      </c>
-      <c r="H33" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B34" s="94"/>
-      <c r="C34" s="96" t="s">
-        <v>52</v>
-      </c>
-      <c r="D34" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="E34" s="52">
-        <v>5</v>
-      </c>
-      <c r="F34" s="38">
-        <v>1</v>
-      </c>
-      <c r="G34" s="38">
-        <v>0</v>
-      </c>
-      <c r="H34" s="39">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B35" s="95"/>
-      <c r="C35" s="98"/>
-      <c r="D35" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="E35" s="51">
-        <v>5</v>
-      </c>
-      <c r="F35" s="40">
-        <v>1</v>
-      </c>
-      <c r="G35" s="40">
-        <v>0</v>
-      </c>
-      <c r="H35" s="41">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B36" s="99" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="100"/>
-      <c r="D36" s="100"/>
-      <c r="E36" s="100"/>
-      <c r="F36" s="100"/>
-      <c r="G36" s="100"/>
-      <c r="H36" s="6">
-        <f>SUM(H12:H35)</f>
-        <v>7868</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B37" s="101" t="s">
-        <v>56</v>
-      </c>
-      <c r="C37" s="102"/>
-      <c r="D37" s="102"/>
-      <c r="E37" s="102"/>
-      <c r="F37" s="102"/>
-      <c r="G37" s="102"/>
-      <c r="H37" s="4">
-        <f>H36/D5</f>
-        <v>983.5</v>
-      </c>
-    </row>
-    <row r="38" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B38" s="101" t="s">
-        <v>57</v>
-      </c>
-      <c r="C38" s="102"/>
-      <c r="D38" s="102"/>
-      <c r="E38" s="102"/>
-      <c r="F38" s="102"/>
-      <c r="G38" s="102"/>
-      <c r="H38" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B39" s="90" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" s="91"/>
-      <c r="D39" s="91"/>
-      <c r="E39" s="91"/>
-      <c r="F39" s="91"/>
-      <c r="G39" s="91"/>
-      <c r="H39" s="5">
-        <f>H37+H38</f>
-        <v>983.5</v>
-      </c>
-    </row>
-    <row r="40" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1"/>
-    <row r="41" spans="2:8" s="32" customFormat="1" ht="16.5" customHeight="1"/>
-    <row r="42" spans="2:8" s="32" customFormat="1" ht="16.5" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:H10"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B26"/>
-    <mergeCell ref="C21:C26"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B27:B35"/>
-    <mergeCell ref="C27:C33"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B38:G38"/>
-  </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:O74"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="20.149999999999999" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="20.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="1.5" style="58" customWidth="1"/>
     <col min="2" max="2" width="9.33203125" style="58" customWidth="1"/>
-    <col min="3" max="3" width="10.08203125" style="58" customWidth="1"/>
+    <col min="3" max="3" width="10" style="58" customWidth="1"/>
     <col min="4" max="16384" width="9" style="58"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="14">
-      <c r="E2" s="143"/>
-      <c r="F2" s="143"/>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
-      <c r="I2" s="143"/>
-      <c r="J2" s="143"/>
-      <c r="K2" s="143"/>
-      <c r="L2" s="143"/>
-      <c r="M2" s="143"/>
-      <c r="N2" s="143"/>
-    </row>
-    <row r="3" spans="2:14" ht="14"/>
-    <row r="4" spans="2:14" ht="14"/>
-    <row r="5" spans="2:14" ht="14">
-      <c r="B5" s="144" t="s">
+    <row r="2" spans="2:14" ht="15">
+      <c r="E2" s="203"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="203"/>
+      <c r="H2" s="203"/>
+      <c r="I2" s="203"/>
+      <c r="J2" s="203"/>
+      <c r="K2" s="203"/>
+      <c r="L2" s="203"/>
+      <c r="M2" s="203"/>
+      <c r="N2" s="203"/>
+    </row>
+    <row r="3" spans="2:14" ht="15"/>
+    <row r="4" spans="2:14" ht="15"/>
+    <row r="5" spans="2:14" ht="15">
+      <c r="B5" s="143" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="144"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="144"/>
-      <c r="H5" s="144"/>
-      <c r="I5" s="144"/>
-      <c r="J5" s="144"/>
-      <c r="K5" s="144"/>
-      <c r="L5" s="144"/>
-      <c r="M5" s="144"/>
-      <c r="N5" s="144"/>
-    </row>
-    <row r="6" spans="2:14" ht="14"/>
-    <row r="7" spans="2:14" ht="14">
-      <c r="B7" s="145" t="s">
+      <c r="C5" s="143"/>
+      <c r="D5" s="143"/>
+      <c r="E5" s="143"/>
+      <c r="F5" s="143"/>
+      <c r="G5" s="143"/>
+      <c r="H5" s="143"/>
+      <c r="I5" s="143"/>
+      <c r="J5" s="143"/>
+      <c r="K5" s="143"/>
+      <c r="L5" s="143"/>
+      <c r="M5" s="143"/>
+      <c r="N5" s="143"/>
+    </row>
+    <row r="6" spans="2:14" ht="15"/>
+    <row r="7" spans="2:14" ht="15">
+      <c r="B7" s="169" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="146"/>
-      <c r="D7" s="147" t="s">
+      <c r="C7" s="171"/>
+      <c r="D7" s="195" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="148"/>
-      <c r="F7" s="148"/>
-      <c r="G7" s="148"/>
-      <c r="H7" s="145" t="s">
+      <c r="E7" s="196"/>
+      <c r="F7" s="196"/>
+      <c r="G7" s="196"/>
+      <c r="H7" s="169" t="s">
         <v>62</v>
       </c>
-      <c r="I7" s="146"/>
-      <c r="J7" s="147" t="s">
+      <c r="I7" s="171"/>
+      <c r="J7" s="195" t="s">
         <v>63</v>
       </c>
-      <c r="K7" s="148"/>
-      <c r="L7" s="148"/>
-      <c r="M7" s="148"/>
-      <c r="N7" s="149"/>
-    </row>
-    <row r="8" spans="2:14" ht="14">
-      <c r="B8" s="145" t="s">
+      <c r="K7" s="196"/>
+      <c r="L7" s="196"/>
+      <c r="M7" s="196"/>
+      <c r="N7" s="197"/>
+    </row>
+    <row r="8" spans="2:14" ht="15">
+      <c r="B8" s="169" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="146"/>
-      <c r="D8" s="147" t="s">
+      <c r="C8" s="171"/>
+      <c r="D8" s="195" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="148"/>
-      <c r="F8" s="148"/>
-      <c r="G8" s="148"/>
-      <c r="H8" s="145" t="s">
+      <c r="E8" s="196"/>
+      <c r="F8" s="196"/>
+      <c r="G8" s="196"/>
+      <c r="H8" s="169" t="s">
         <v>66</v>
       </c>
-      <c r="I8" s="146"/>
-      <c r="J8" s="147">
+      <c r="I8" s="171"/>
+      <c r="J8" s="195">
         <v>8</v>
       </c>
-      <c r="K8" s="148"/>
-      <c r="L8" s="148"/>
-      <c r="M8" s="148"/>
-      <c r="N8" s="149"/>
-    </row>
-    <row r="9" spans="2:14" ht="14">
-      <c r="B9" s="155" t="s">
+      <c r="K8" s="196"/>
+      <c r="L8" s="196"/>
+      <c r="M8" s="196"/>
+      <c r="N8" s="197"/>
+    </row>
+    <row r="9" spans="2:14" ht="15">
+      <c r="B9" s="199" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="156"/>
-      <c r="D9" s="145" t="s">
+      <c r="C9" s="200"/>
+      <c r="D9" s="169" t="s">
         <v>68</v>
       </c>
-      <c r="E9" s="159"/>
-      <c r="F9" s="146"/>
-      <c r="G9" s="145" t="s">
+      <c r="E9" s="170"/>
+      <c r="F9" s="171"/>
+      <c r="G9" s="169" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="159"/>
-      <c r="I9" s="146"/>
-      <c r="J9" s="145" t="s">
+      <c r="H9" s="170"/>
+      <c r="I9" s="171"/>
+      <c r="J9" s="169" t="s">
         <v>70</v>
       </c>
-      <c r="K9" s="159"/>
-      <c r="L9" s="146"/>
-      <c r="M9" s="145" t="s">
+      <c r="K9" s="170"/>
+      <c r="L9" s="171"/>
+      <c r="M9" s="169" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="146"/>
-    </row>
-    <row r="10" spans="2:14" ht="14">
-      <c r="B10" s="157"/>
-      <c r="C10" s="158"/>
-      <c r="D10" s="147">
+      <c r="N9" s="171"/>
+    </row>
+    <row r="10" spans="2:14" ht="15">
+      <c r="B10" s="201"/>
+      <c r="C10" s="202"/>
+      <c r="D10" s="195">
         <v>8</v>
       </c>
-      <c r="E10" s="148"/>
-      <c r="F10" s="149"/>
-      <c r="G10" s="147" t="s">
+      <c r="E10" s="196"/>
+      <c r="F10" s="197"/>
+      <c r="G10" s="195" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="148"/>
-      <c r="I10" s="149"/>
-      <c r="J10" s="147"/>
-      <c r="K10" s="148"/>
-      <c r="L10" s="149"/>
-      <c r="M10" s="150" t="s">
+      <c r="H10" s="196"/>
+      <c r="I10" s="197"/>
+      <c r="J10" s="195"/>
+      <c r="K10" s="196"/>
+      <c r="L10" s="197"/>
+      <c r="M10" s="181" t="s">
         <v>72</v>
       </c>
-      <c r="N10" s="151"/>
-    </row>
-    <row r="11" spans="2:14" ht="14">
-      <c r="B11" s="147"/>
-      <c r="C11" s="148"/>
-      <c r="D11" s="148"/>
-      <c r="E11" s="148"/>
-      <c r="F11" s="148"/>
-      <c r="G11" s="148"/>
-      <c r="H11" s="148"/>
-      <c r="I11" s="148"/>
-      <c r="J11" s="148"/>
-      <c r="K11" s="148"/>
-      <c r="L11" s="148"/>
-      <c r="M11" s="148"/>
-      <c r="N11" s="149"/>
-    </row>
-    <row r="12" spans="2:14" ht="14">
-      <c r="B12" s="152" t="s">
+      <c r="N10" s="183"/>
+    </row>
+    <row r="11" spans="2:14" ht="15">
+      <c r="B11" s="195"/>
+      <c r="C11" s="196"/>
+      <c r="D11" s="196"/>
+      <c r="E11" s="196"/>
+      <c r="F11" s="196"/>
+      <c r="G11" s="196"/>
+      <c r="H11" s="196"/>
+      <c r="I11" s="196"/>
+      <c r="J11" s="196"/>
+      <c r="K11" s="196"/>
+      <c r="L11" s="196"/>
+      <c r="M11" s="196"/>
+      <c r="N11" s="197"/>
+    </row>
+    <row r="12" spans="2:14" ht="15">
+      <c r="B12" s="186" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="153"/>
-      <c r="D12" s="152" t="s">
+      <c r="C12" s="187"/>
+      <c r="D12" s="186" t="s">
         <v>74</v>
       </c>
-      <c r="E12" s="154"/>
-      <c r="F12" s="154"/>
-      <c r="G12" s="154"/>
-      <c r="H12" s="154"/>
-      <c r="I12" s="154"/>
-      <c r="J12" s="154"/>
-      <c r="K12" s="154"/>
-      <c r="L12" s="153"/>
-      <c r="M12" s="152" t="s">
+      <c r="E12" s="198"/>
+      <c r="F12" s="198"/>
+      <c r="G12" s="198"/>
+      <c r="H12" s="198"/>
+      <c r="I12" s="198"/>
+      <c r="J12" s="198"/>
+      <c r="K12" s="198"/>
+      <c r="L12" s="187"/>
+      <c r="M12" s="186" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="153"/>
-    </row>
-    <row r="13" spans="2:14" ht="14">
-      <c r="B13" s="160" t="s">
+      <c r="N12" s="187"/>
+    </row>
+    <row r="13" spans="2:14" ht="15">
+      <c r="B13" s="188" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="161"/>
-      <c r="D13" s="152" t="s">
+      <c r="C13" s="189"/>
+      <c r="D13" s="186" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="153"/>
-      <c r="F13" s="150" t="s">
+      <c r="E13" s="187"/>
+      <c r="F13" s="181" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="164"/>
-      <c r="H13" s="151"/>
+      <c r="G13" s="182"/>
+      <c r="H13" s="183"/>
       <c r="I13" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="J13" s="150" t="s">
+      <c r="J13" s="181" t="s">
         <v>79</v>
       </c>
-      <c r="K13" s="164"/>
-      <c r="L13" s="151"/>
-      <c r="M13" s="165"/>
-      <c r="N13" s="165"/>
-    </row>
-    <row r="14" spans="2:14" ht="14">
-      <c r="B14" s="162"/>
-      <c r="C14" s="163"/>
-      <c r="D14" s="152" t="s">
+      <c r="K13" s="182"/>
+      <c r="L13" s="183"/>
+      <c r="M13" s="192"/>
+      <c r="N13" s="192"/>
+    </row>
+    <row r="14" spans="2:14" ht="15">
+      <c r="B14" s="190"/>
+      <c r="C14" s="191"/>
+      <c r="D14" s="186" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="153"/>
-      <c r="F14" s="150" t="s">
+      <c r="E14" s="187"/>
+      <c r="F14" s="181" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="164"/>
-      <c r="H14" s="151"/>
+      <c r="G14" s="182"/>
+      <c r="H14" s="183"/>
       <c r="I14" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="J14" s="150" t="s">
+      <c r="J14" s="181" t="s">
         <v>12</v>
       </c>
-      <c r="K14" s="164"/>
-      <c r="L14" s="151"/>
-      <c r="M14" s="166" t="s">
+      <c r="K14" s="182"/>
+      <c r="L14" s="183"/>
+      <c r="M14" s="193" t="s">
         <v>82</v>
       </c>
-      <c r="N14" s="167"/>
-    </row>
-    <row r="15" spans="2:14" ht="14">
-      <c r="B15" s="168" t="s">
+      <c r="N14" s="194"/>
+    </row>
+    <row r="15" spans="2:14" ht="15">
+      <c r="B15" s="178" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="169"/>
-      <c r="D15" s="152" t="s">
+      <c r="C15" s="179"/>
+      <c r="D15" s="186" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="153"/>
-      <c r="F15" s="150" t="s">
+      <c r="E15" s="187"/>
+      <c r="F15" s="181" t="s">
         <v>85</v>
       </c>
-      <c r="G15" s="164"/>
-      <c r="H15" s="151"/>
+      <c r="G15" s="182"/>
+      <c r="H15" s="183"/>
       <c r="I15" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="J15" s="150" t="s">
+      <c r="J15" s="181" t="s">
         <v>87</v>
       </c>
-      <c r="K15" s="164"/>
-      <c r="L15" s="151"/>
-      <c r="M15" s="170"/>
-      <c r="N15" s="171"/>
-    </row>
-    <row r="16" spans="2:14" ht="14">
-      <c r="B16" s="168" t="s">
+      <c r="K15" s="182"/>
+      <c r="L15" s="183"/>
+      <c r="M15" s="176"/>
+      <c r="N15" s="177"/>
+    </row>
+    <row r="16" spans="2:14" ht="15">
+      <c r="B16" s="178" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="169"/>
-      <c r="D16" s="150" t="s">
+      <c r="C16" s="179"/>
+      <c r="D16" s="181" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="164"/>
-      <c r="F16" s="164" t="s">
+      <c r="E16" s="182"/>
+      <c r="F16" s="182" t="s">
         <v>89</v>
       </c>
-      <c r="G16" s="164"/>
-      <c r="H16" s="164" t="s">
+      <c r="G16" s="182"/>
+      <c r="H16" s="182" t="s">
         <v>90</v>
       </c>
-      <c r="I16" s="164"/>
-      <c r="J16" s="164" t="s">
+      <c r="I16" s="182"/>
+      <c r="J16" s="182" t="s">
         <v>91</v>
       </c>
-      <c r="K16" s="164"/>
+      <c r="K16" s="182"/>
       <c r="L16" s="60"/>
-      <c r="M16" s="172" t="s">
+      <c r="M16" s="184" t="s">
         <v>92</v>
       </c>
-      <c r="N16" s="173"/>
-    </row>
-    <row r="17" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B17" s="168" t="s">
+      <c r="N16" s="185"/>
+    </row>
+    <row r="17" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B17" s="178" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="169"/>
-      <c r="D17" s="150" t="s">
+      <c r="C17" s="179"/>
+      <c r="D17" s="181" t="s">
         <v>94</v>
       </c>
-      <c r="E17" s="164"/>
-      <c r="F17" s="164" t="s">
+      <c r="E17" s="182"/>
+      <c r="F17" s="182" t="s">
         <v>95</v>
       </c>
-      <c r="G17" s="164"/>
+      <c r="G17" s="182"/>
       <c r="H17" s="61"/>
       <c r="I17" s="61"/>
       <c r="J17" s="61"/>
       <c r="K17" s="61"/>
       <c r="L17" s="60"/>
-      <c r="M17" s="172" t="s">
+      <c r="M17" s="184" t="s">
         <v>92</v>
       </c>
-      <c r="N17" s="173"/>
-    </row>
-    <row r="18" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B18" s="168" t="s">
+      <c r="N17" s="185"/>
+    </row>
+    <row r="18" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B18" s="178" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="169"/>
-      <c r="D18" s="150" t="s">
+      <c r="C18" s="179"/>
+      <c r="D18" s="181" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="164"/>
-      <c r="F18" s="164" t="s">
+      <c r="E18" s="182"/>
+      <c r="F18" s="182" t="s">
         <v>95</v>
       </c>
-      <c r="G18" s="164"/>
+      <c r="G18" s="182"/>
       <c r="H18" s="174" t="s">
         <v>97</v>
       </c>
@@ -3834,64 +3061,64 @@
       <c r="J18" s="174"/>
       <c r="K18" s="174"/>
       <c r="L18" s="175"/>
-      <c r="M18" s="170"/>
-      <c r="N18" s="171"/>
-    </row>
-    <row r="19" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B19" s="168" t="s">
+      <c r="M18" s="176"/>
+      <c r="N18" s="177"/>
+    </row>
+    <row r="19" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B19" s="178" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="169"/>
-      <c r="D19" s="150" t="s">
+      <c r="C19" s="179"/>
+      <c r="D19" s="181" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="164"/>
-      <c r="F19" s="164" t="s">
+      <c r="E19" s="182"/>
+      <c r="F19" s="182" t="s">
         <v>100</v>
       </c>
-      <c r="G19" s="164"/>
-      <c r="H19" s="164"/>
-      <c r="I19" s="164"/>
-      <c r="J19" s="164"/>
-      <c r="K19" s="164"/>
-      <c r="L19" s="151"/>
-      <c r="M19" s="170"/>
-      <c r="N19" s="171"/>
-    </row>
-    <row r="20" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B20" s="168" t="s">
+      <c r="G19" s="182"/>
+      <c r="H19" s="182"/>
+      <c r="I19" s="182"/>
+      <c r="J19" s="182"/>
+      <c r="K19" s="182"/>
+      <c r="L19" s="183"/>
+      <c r="M19" s="176"/>
+      <c r="N19" s="177"/>
+    </row>
+    <row r="20" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B20" s="178" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="169"/>
-      <c r="D20" s="150" t="s">
+      <c r="C20" s="179"/>
+      <c r="D20" s="181" t="s">
         <v>99</v>
       </c>
-      <c r="E20" s="164"/>
-      <c r="F20" s="164" t="s">
+      <c r="E20" s="182"/>
+      <c r="F20" s="182" t="s">
         <v>100</v>
       </c>
-      <c r="G20" s="164"/>
+      <c r="G20" s="182"/>
       <c r="H20" s="174"/>
       <c r="I20" s="174"/>
       <c r="J20" s="174"/>
       <c r="K20" s="174"/>
       <c r="L20" s="175"/>
-      <c r="M20" s="170"/>
-      <c r="N20" s="171"/>
-    </row>
-    <row r="21" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B21" s="168" t="s">
+      <c r="M20" s="176"/>
+      <c r="N20" s="177"/>
+    </row>
+    <row r="21" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B21" s="178" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="169"/>
-      <c r="D21" s="150" t="s">
+      <c r="C21" s="179"/>
+      <c r="D21" s="181" t="s">
         <v>99</v>
       </c>
-      <c r="E21" s="164"/>
-      <c r="F21" s="164" t="s">
+      <c r="E21" s="182"/>
+      <c r="F21" s="182" t="s">
         <v>100</v>
       </c>
-      <c r="G21" s="164"/>
+      <c r="G21" s="182"/>
       <c r="H21" s="174" t="s">
         <v>12</v>
       </c>
@@ -3899,22 +3126,22 @@
       <c r="J21" s="174"/>
       <c r="K21" s="174"/>
       <c r="L21" s="175"/>
-      <c r="M21" s="170"/>
-      <c r="N21" s="171"/>
-    </row>
-    <row r="22" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B22" s="168" t="s">
+      <c r="M21" s="176"/>
+      <c r="N21" s="177"/>
+    </row>
+    <row r="22" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B22" s="178" t="s">
         <v>103</v>
       </c>
-      <c r="C22" s="169"/>
-      <c r="D22" s="150" t="s">
+      <c r="C22" s="179"/>
+      <c r="D22" s="181" t="s">
         <v>94</v>
       </c>
-      <c r="E22" s="164"/>
-      <c r="F22" s="164" t="s">
+      <c r="E22" s="182"/>
+      <c r="F22" s="182" t="s">
         <v>95</v>
       </c>
-      <c r="G22" s="164"/>
+      <c r="G22" s="182"/>
       <c r="H22" s="174" t="s">
         <v>104</v>
       </c>
@@ -3922,22 +3149,22 @@
       <c r="J22" s="174"/>
       <c r="K22" s="174"/>
       <c r="L22" s="175"/>
-      <c r="M22" s="170"/>
-      <c r="N22" s="171"/>
-    </row>
-    <row r="23" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B23" s="168" t="s">
+      <c r="M22" s="176"/>
+      <c r="N22" s="177"/>
+    </row>
+    <row r="23" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B23" s="178" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="169"/>
-      <c r="D23" s="150" t="s">
+      <c r="C23" s="179"/>
+      <c r="D23" s="181" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="164"/>
-      <c r="F23" s="164" t="s">
+      <c r="E23" s="182"/>
+      <c r="F23" s="182" t="s">
         <v>95</v>
       </c>
-      <c r="G23" s="164"/>
+      <c r="G23" s="182"/>
       <c r="H23" s="174" t="s">
         <v>106</v>
       </c>
@@ -3945,15 +3172,15 @@
       <c r="J23" s="174"/>
       <c r="K23" s="174"/>
       <c r="L23" s="175"/>
-      <c r="M23" s="170"/>
-      <c r="N23" s="171"/>
-    </row>
-    <row r="24" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B24" s="168" t="s">
+      <c r="M23" s="176"/>
+      <c r="N23" s="177"/>
+    </row>
+    <row r="24" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B24" s="178" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="169"/>
-      <c r="D24" s="177" t="s">
+      <c r="C24" s="179"/>
+      <c r="D24" s="173" t="s">
         <v>108</v>
       </c>
       <c r="E24" s="174"/>
@@ -3964,15 +3191,15 @@
       <c r="J24" s="174"/>
       <c r="K24" s="174"/>
       <c r="L24" s="175"/>
-      <c r="M24" s="170"/>
-      <c r="N24" s="171"/>
-    </row>
-    <row r="25" spans="2:15" ht="20.149999999999999" customHeight="1">
-      <c r="B25" s="176" t="s">
+      <c r="M24" s="176"/>
+      <c r="N24" s="177"/>
+    </row>
+    <row r="25" spans="2:15" ht="20.25" customHeight="1">
+      <c r="B25" s="172" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="176"/>
-      <c r="D25" s="177" t="s">
+      <c r="C25" s="172"/>
+      <c r="D25" s="173" t="s">
         <v>110</v>
       </c>
       <c r="E25" s="174"/>
@@ -3983,15 +3210,15 @@
       <c r="J25" s="174"/>
       <c r="K25" s="174"/>
       <c r="L25" s="175"/>
-      <c r="M25" s="170"/>
-      <c r="N25" s="171"/>
+      <c r="M25" s="176"/>
+      <c r="N25" s="177"/>
     </row>
     <row r="26" spans="2:15" ht="81.75" customHeight="1">
-      <c r="B26" s="168" t="s">
+      <c r="B26" s="178" t="s">
         <v>111</v>
       </c>
-      <c r="C26" s="169"/>
-      <c r="D26" s="178" t="s">
+      <c r="C26" s="179"/>
+      <c r="D26" s="180" t="s">
         <v>112</v>
       </c>
       <c r="E26" s="174"/>
@@ -4006,11 +3233,11 @@
       <c r="N26" s="63"/>
     </row>
     <row r="27" spans="2:15" ht="51" customHeight="1">
-      <c r="B27" s="176" t="s">
+      <c r="B27" s="172" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="176"/>
-      <c r="D27" s="178" t="s">
+      <c r="C27" s="172"/>
+      <c r="D27" s="180" t="s">
         <v>114</v>
       </c>
       <c r="E27" s="174"/>
@@ -4021,11 +3248,11 @@
       <c r="J27" s="174"/>
       <c r="K27" s="174"/>
       <c r="L27" s="175"/>
-      <c r="M27" s="170"/>
-      <c r="N27" s="171"/>
+      <c r="M27" s="176"/>
+      <c r="N27" s="177"/>
     </row>
     <row r="28" spans="2:15" ht="11.25" customHeight="1"/>
-    <row r="29" spans="2:15" ht="20.149999999999999" customHeight="1">
+    <row r="29" spans="2:15" ht="20.25" customHeight="1">
       <c r="B29" s="64" t="s">
         <v>115</v>
       </c>
@@ -4038,21 +3265,21 @@
       <c r="E29" s="64" t="s">
         <v>118</v>
       </c>
-      <c r="F29" s="145" t="s">
+      <c r="F29" s="169" t="s">
         <v>119</v>
       </c>
-      <c r="G29" s="159"/>
-      <c r="H29" s="159"/>
-      <c r="I29" s="159"/>
-      <c r="J29" s="159"/>
-      <c r="K29" s="159"/>
-      <c r="L29" s="146"/>
-      <c r="M29" s="145" t="s">
+      <c r="G29" s="170"/>
+      <c r="H29" s="170"/>
+      <c r="I29" s="170"/>
+      <c r="J29" s="170"/>
+      <c r="K29" s="170"/>
+      <c r="L29" s="171"/>
+      <c r="M29" s="169" t="s">
         <v>45</v>
       </c>
-      <c r="N29" s="146"/>
-    </row>
-    <row r="30" spans="2:15" s="69" customFormat="1" ht="20.149999999999999" customHeight="1">
+      <c r="N29" s="171"/>
+    </row>
+    <row r="30" spans="2:15" s="69" customFormat="1" ht="20.25" customHeight="1">
       <c r="B30" s="65" t="s">
         <v>120</v>
       </c>
@@ -4065,20 +3292,20 @@
       <c r="E30" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="187" t="s">
+      <c r="F30" s="161" t="s">
         <v>122</v>
       </c>
-      <c r="G30" s="188"/>
-      <c r="H30" s="188"/>
-      <c r="I30" s="188"/>
-      <c r="J30" s="188"/>
-      <c r="K30" s="188"/>
-      <c r="L30" s="189"/>
-      <c r="M30" s="190"/>
-      <c r="N30" s="191"/>
+      <c r="G30" s="162"/>
+      <c r="H30" s="162"/>
+      <c r="I30" s="162"/>
+      <c r="J30" s="162"/>
+      <c r="K30" s="162"/>
+      <c r="L30" s="163"/>
+      <c r="M30" s="164"/>
+      <c r="N30" s="165"/>
       <c r="O30" s="68"/>
     </row>
-    <row r="31" spans="2:15" s="69" customFormat="1" ht="20.149999999999999" customHeight="1">
+    <row r="31" spans="2:15" s="69" customFormat="1" ht="20.25" customHeight="1">
       <c r="B31" s="66"/>
       <c r="C31" s="66" t="s">
         <v>123</v>
@@ -4087,70 +3314,70 @@
       <c r="E31" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="F31" s="179" t="s">
+      <c r="F31" s="159" t="s">
         <v>124</v>
       </c>
-      <c r="G31" s="180"/>
-      <c r="H31" s="180"/>
-      <c r="I31" s="180"/>
-      <c r="J31" s="180"/>
-      <c r="K31" s="180"/>
-      <c r="L31" s="181"/>
-      <c r="M31" s="182"/>
-      <c r="N31" s="183"/>
-    </row>
-    <row r="32" spans="2:15" s="69" customFormat="1" ht="20.149999999999999" customHeight="1">
+      <c r="G31" s="147"/>
+      <c r="H31" s="147"/>
+      <c r="I31" s="147"/>
+      <c r="J31" s="147"/>
+      <c r="K31" s="147"/>
+      <c r="L31" s="160"/>
+      <c r="M31" s="149"/>
+      <c r="N31" s="153"/>
+    </row>
+    <row r="32" spans="2:15" s="69" customFormat="1" ht="20.25" customHeight="1">
       <c r="B32" s="66"/>
       <c r="C32" s="66"/>
       <c r="D32" s="66"/>
       <c r="E32" s="67"/>
-      <c r="F32" s="179" t="s">
+      <c r="F32" s="159" t="s">
         <v>125</v>
       </c>
-      <c r="G32" s="180"/>
-      <c r="H32" s="180"/>
-      <c r="I32" s="180"/>
-      <c r="J32" s="180"/>
-      <c r="K32" s="180"/>
-      <c r="L32" s="181"/>
-      <c r="M32" s="182" t="s">
+      <c r="G32" s="147"/>
+      <c r="H32" s="147"/>
+      <c r="I32" s="147"/>
+      <c r="J32" s="147"/>
+      <c r="K32" s="147"/>
+      <c r="L32" s="160"/>
+      <c r="M32" s="149" t="s">
         <v>12</v>
       </c>
-      <c r="N32" s="183"/>
+      <c r="N32" s="153"/>
     </row>
     <row r="33" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B33" s="66"/>
       <c r="C33" s="66"/>
       <c r="D33" s="66"/>
       <c r="E33" s="66"/>
-      <c r="F33" s="179" t="s">
+      <c r="F33" s="159" t="s">
         <v>126</v>
       </c>
-      <c r="G33" s="180"/>
-      <c r="H33" s="180"/>
-      <c r="I33" s="180"/>
-      <c r="J33" s="180"/>
-      <c r="K33" s="180"/>
-      <c r="L33" s="181"/>
-      <c r="M33" s="182"/>
-      <c r="N33" s="183"/>
+      <c r="G33" s="147"/>
+      <c r="H33" s="147"/>
+      <c r="I33" s="147"/>
+      <c r="J33" s="147"/>
+      <c r="K33" s="147"/>
+      <c r="L33" s="160"/>
+      <c r="M33" s="149"/>
+      <c r="N33" s="153"/>
     </row>
     <row r="34" spans="2:14" s="69" customFormat="1" ht="13">
-      <c r="B34" s="184" t="s">
+      <c r="B34" s="166" t="s">
         <v>127</v>
       </c>
-      <c r="C34" s="185"/>
-      <c r="D34" s="185"/>
-      <c r="E34" s="185"/>
-      <c r="F34" s="185"/>
-      <c r="G34" s="185"/>
-      <c r="H34" s="185"/>
-      <c r="I34" s="185"/>
-      <c r="J34" s="185"/>
-      <c r="K34" s="185"/>
-      <c r="L34" s="185"/>
-      <c r="M34" s="185"/>
-      <c r="N34" s="186"/>
+      <c r="C34" s="167"/>
+      <c r="D34" s="167"/>
+      <c r="E34" s="167"/>
+      <c r="F34" s="167"/>
+      <c r="G34" s="167"/>
+      <c r="H34" s="167"/>
+      <c r="I34" s="167"/>
+      <c r="J34" s="167"/>
+      <c r="K34" s="167"/>
+      <c r="L34" s="167"/>
+      <c r="M34" s="167"/>
+      <c r="N34" s="168"/>
     </row>
     <row r="35" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B35" s="65" t="s">
@@ -4161,19 +3388,19 @@
         <v>129</v>
       </c>
       <c r="E35" s="67"/>
-      <c r="F35" s="187" t="s">
+      <c r="F35" s="161" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="188"/>
-      <c r="H35" s="188"/>
-      <c r="I35" s="188"/>
-      <c r="J35" s="188"/>
-      <c r="K35" s="188"/>
-      <c r="L35" s="189"/>
-      <c r="M35" s="190" t="s">
+      <c r="G35" s="162"/>
+      <c r="H35" s="162"/>
+      <c r="I35" s="162"/>
+      <c r="J35" s="162"/>
+      <c r="K35" s="162"/>
+      <c r="L35" s="163"/>
+      <c r="M35" s="164" t="s">
         <v>131</v>
       </c>
-      <c r="N35" s="191"/>
+      <c r="N35" s="165"/>
     </row>
     <row r="36" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B36" s="70"/>
@@ -4182,17 +3409,17 @@
       </c>
       <c r="D36" s="66"/>
       <c r="E36" s="67"/>
-      <c r="F36" s="179" t="s">
+      <c r="F36" s="159" t="s">
         <v>133</v>
       </c>
-      <c r="G36" s="180"/>
-      <c r="H36" s="180"/>
-      <c r="I36" s="180"/>
-      <c r="J36" s="180"/>
-      <c r="K36" s="180"/>
-      <c r="L36" s="181"/>
-      <c r="M36" s="182"/>
-      <c r="N36" s="183"/>
+      <c r="G36" s="147"/>
+      <c r="H36" s="147"/>
+      <c r="I36" s="147"/>
+      <c r="J36" s="147"/>
+      <c r="K36" s="147"/>
+      <c r="L36" s="160"/>
+      <c r="M36" s="149"/>
+      <c r="N36" s="153"/>
     </row>
     <row r="37" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B37" s="66"/>
@@ -4201,19 +3428,19 @@
       </c>
       <c r="D37" s="66"/>
       <c r="E37" s="67"/>
-      <c r="F37" s="179" t="s">
+      <c r="F37" s="159" t="s">
         <v>134</v>
       </c>
-      <c r="G37" s="180"/>
-      <c r="H37" s="180"/>
-      <c r="I37" s="180"/>
-      <c r="J37" s="180"/>
-      <c r="K37" s="180"/>
-      <c r="L37" s="181"/>
-      <c r="M37" s="182" t="s">
+      <c r="G37" s="147"/>
+      <c r="H37" s="147"/>
+      <c r="I37" s="147"/>
+      <c r="J37" s="147"/>
+      <c r="K37" s="147"/>
+      <c r="L37" s="160"/>
+      <c r="M37" s="149" t="s">
         <v>135</v>
       </c>
-      <c r="N37" s="183"/>
+      <c r="N37" s="153"/>
     </row>
     <row r="38" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B38" s="70"/>
@@ -4222,51 +3449,51 @@
       </c>
       <c r="D38" s="66"/>
       <c r="E38" s="66"/>
-      <c r="F38" s="179" t="s">
+      <c r="F38" s="159" t="s">
         <v>136</v>
       </c>
-      <c r="G38" s="180"/>
-      <c r="H38" s="180"/>
-      <c r="I38" s="180"/>
-      <c r="J38" s="180"/>
-      <c r="K38" s="180"/>
-      <c r="L38" s="181"/>
-      <c r="M38" s="182"/>
-      <c r="N38" s="183"/>
+      <c r="G38" s="147"/>
+      <c r="H38" s="147"/>
+      <c r="I38" s="147"/>
+      <c r="J38" s="147"/>
+      <c r="K38" s="147"/>
+      <c r="L38" s="160"/>
+      <c r="M38" s="149"/>
+      <c r="N38" s="153"/>
     </row>
     <row r="39" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B39" s="70"/>
       <c r="C39" s="66"/>
       <c r="D39" s="66"/>
       <c r="E39" s="66"/>
-      <c r="F39" s="179" t="s">
+      <c r="F39" s="159" t="s">
         <v>137</v>
       </c>
-      <c r="G39" s="180"/>
-      <c r="H39" s="180"/>
-      <c r="I39" s="180"/>
-      <c r="J39" s="180"/>
-      <c r="K39" s="180"/>
-      <c r="L39" s="181"/>
-      <c r="M39" s="182" t="s">
+      <c r="G39" s="147"/>
+      <c r="H39" s="147"/>
+      <c r="I39" s="147"/>
+      <c r="J39" s="147"/>
+      <c r="K39" s="147"/>
+      <c r="L39" s="160"/>
+      <c r="M39" s="149" t="s">
         <v>138</v>
       </c>
-      <c r="N39" s="183"/>
+      <c r="N39" s="153"/>
     </row>
     <row r="40" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B40" s="70"/>
       <c r="C40" s="66"/>
       <c r="D40" s="66"/>
       <c r="E40" s="66"/>
-      <c r="F40" s="179" t="s">
+      <c r="F40" s="159" t="s">
         <v>139</v>
       </c>
-      <c r="G40" s="180"/>
-      <c r="H40" s="180"/>
-      <c r="I40" s="180"/>
-      <c r="J40" s="180"/>
-      <c r="K40" s="180"/>
-      <c r="L40" s="181"/>
+      <c r="G40" s="147"/>
+      <c r="H40" s="147"/>
+      <c r="I40" s="147"/>
+      <c r="J40" s="147"/>
+      <c r="K40" s="147"/>
+      <c r="L40" s="160"/>
       <c r="M40" s="71"/>
       <c r="N40" s="72"/>
     </row>
@@ -4277,19 +3504,19 @@
       </c>
       <c r="D41" s="66"/>
       <c r="E41" s="66"/>
-      <c r="F41" s="179" t="s">
+      <c r="F41" s="159" t="s">
         <v>140</v>
       </c>
-      <c r="G41" s="180"/>
-      <c r="H41" s="180"/>
-      <c r="I41" s="180"/>
-      <c r="J41" s="180"/>
-      <c r="K41" s="180"/>
-      <c r="L41" s="181"/>
-      <c r="M41" s="182" t="s">
+      <c r="G41" s="147"/>
+      <c r="H41" s="147"/>
+      <c r="I41" s="147"/>
+      <c r="J41" s="147"/>
+      <c r="K41" s="147"/>
+      <c r="L41" s="160"/>
+      <c r="M41" s="149" t="s">
         <v>12</v>
       </c>
-      <c r="N41" s="183"/>
+      <c r="N41" s="153"/>
     </row>
     <row r="42" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B42" s="66"/>
@@ -4298,34 +3525,34 @@
       </c>
       <c r="D42" s="66"/>
       <c r="E42" s="66"/>
-      <c r="F42" s="179" t="s">
+      <c r="F42" s="159" t="s">
         <v>141</v>
       </c>
-      <c r="G42" s="180"/>
-      <c r="H42" s="180"/>
-      <c r="I42" s="180"/>
-      <c r="J42" s="180"/>
-      <c r="K42" s="180"/>
-      <c r="L42" s="181"/>
-      <c r="M42" s="182"/>
-      <c r="N42" s="183"/>
+      <c r="G42" s="147"/>
+      <c r="H42" s="147"/>
+      <c r="I42" s="147"/>
+      <c r="J42" s="147"/>
+      <c r="K42" s="147"/>
+      <c r="L42" s="160"/>
+      <c r="M42" s="149"/>
+      <c r="N42" s="153"/>
     </row>
     <row r="43" spans="2:14" s="69" customFormat="1" ht="13">
-      <c r="B43" s="184" t="s">
+      <c r="B43" s="166" t="s">
         <v>127</v>
       </c>
-      <c r="C43" s="185"/>
-      <c r="D43" s="185"/>
-      <c r="E43" s="185"/>
-      <c r="F43" s="185"/>
-      <c r="G43" s="185"/>
-      <c r="H43" s="185"/>
-      <c r="I43" s="185"/>
-      <c r="J43" s="185"/>
-      <c r="K43" s="185"/>
-      <c r="L43" s="185"/>
-      <c r="M43" s="185"/>
-      <c r="N43" s="186"/>
+      <c r="C43" s="167"/>
+      <c r="D43" s="167"/>
+      <c r="E43" s="167"/>
+      <c r="F43" s="167"/>
+      <c r="G43" s="167"/>
+      <c r="H43" s="167"/>
+      <c r="I43" s="167"/>
+      <c r="J43" s="167"/>
+      <c r="K43" s="167"/>
+      <c r="L43" s="167"/>
+      <c r="M43" s="167"/>
+      <c r="N43" s="168"/>
     </row>
     <row r="44" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B44" s="65" t="s">
@@ -4338,19 +3565,19 @@
         <v>129</v>
       </c>
       <c r="E44" s="67"/>
-      <c r="F44" s="187" t="s">
+      <c r="F44" s="161" t="s">
         <v>130</v>
       </c>
-      <c r="G44" s="188"/>
-      <c r="H44" s="188"/>
-      <c r="I44" s="188"/>
-      <c r="J44" s="188"/>
-      <c r="K44" s="188"/>
-      <c r="L44" s="189"/>
-      <c r="M44" s="190" t="s">
+      <c r="G44" s="162"/>
+      <c r="H44" s="162"/>
+      <c r="I44" s="162"/>
+      <c r="J44" s="162"/>
+      <c r="K44" s="162"/>
+      <c r="L44" s="163"/>
+      <c r="M44" s="164" t="s">
         <v>131</v>
       </c>
-      <c r="N44" s="191"/>
+      <c r="N44" s="165"/>
     </row>
     <row r="45" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B45" s="70"/>
@@ -4359,53 +3586,53 @@
       </c>
       <c r="D45" s="66"/>
       <c r="E45" s="67"/>
-      <c r="F45" s="179" t="s">
+      <c r="F45" s="159" t="s">
         <v>143</v>
       </c>
-      <c r="G45" s="180"/>
-      <c r="H45" s="180"/>
-      <c r="I45" s="180"/>
-      <c r="J45" s="180"/>
-      <c r="K45" s="180"/>
-      <c r="L45" s="181"/>
-      <c r="M45" s="182"/>
-      <c r="N45" s="183"/>
+      <c r="G45" s="147"/>
+      <c r="H45" s="147"/>
+      <c r="I45" s="147"/>
+      <c r="J45" s="147"/>
+      <c r="K45" s="147"/>
+      <c r="L45" s="160"/>
+      <c r="M45" s="149"/>
+      <c r="N45" s="153"/>
     </row>
     <row r="46" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B46" s="66"/>
       <c r="C46" s="66"/>
       <c r="D46" s="66"/>
       <c r="E46" s="67"/>
-      <c r="F46" s="179" t="s">
+      <c r="F46" s="159" t="s">
         <v>144</v>
       </c>
-      <c r="G46" s="180"/>
-      <c r="H46" s="180"/>
-      <c r="I46" s="180"/>
-      <c r="J46" s="180"/>
-      <c r="K46" s="180"/>
-      <c r="L46" s="181"/>
-      <c r="M46" s="182" t="s">
+      <c r="G46" s="147"/>
+      <c r="H46" s="147"/>
+      <c r="I46" s="147"/>
+      <c r="J46" s="147"/>
+      <c r="K46" s="147"/>
+      <c r="L46" s="160"/>
+      <c r="M46" s="149" t="s">
         <v>145</v>
       </c>
-      <c r="N46" s="183"/>
+      <c r="N46" s="153"/>
     </row>
     <row r="47" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B47" s="66"/>
       <c r="C47" s="66"/>
       <c r="D47" s="66"/>
       <c r="E47" s="67"/>
-      <c r="F47" s="179" t="s">
+      <c r="F47" s="159" t="s">
         <v>146</v>
       </c>
-      <c r="G47" s="180"/>
-      <c r="H47" s="180"/>
-      <c r="I47" s="180"/>
-      <c r="J47" s="180"/>
-      <c r="K47" s="180"/>
-      <c r="L47" s="181"/>
-      <c r="M47" s="182"/>
-      <c r="N47" s="183"/>
+      <c r="G47" s="147"/>
+      <c r="H47" s="147"/>
+      <c r="I47" s="147"/>
+      <c r="J47" s="147"/>
+      <c r="K47" s="147"/>
+      <c r="L47" s="160"/>
+      <c r="M47" s="149"/>
+      <c r="N47" s="153"/>
     </row>
     <row r="48" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B48" s="66"/>
@@ -4421,46 +3648,46 @@
       <c r="J48" s="74"/>
       <c r="K48" s="74"/>
       <c r="L48" s="75"/>
-      <c r="M48" s="182" t="s">
+      <c r="M48" s="149" t="s">
         <v>148</v>
       </c>
-      <c r="N48" s="183"/>
+      <c r="N48" s="153"/>
     </row>
     <row r="49" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B49" s="66"/>
       <c r="C49" s="66"/>
       <c r="D49" s="66"/>
       <c r="E49" s="66"/>
-      <c r="F49" s="179" t="s">
+      <c r="F49" s="159" t="s">
         <v>141</v>
       </c>
-      <c r="G49" s="180"/>
-      <c r="H49" s="180"/>
-      <c r="I49" s="180"/>
-      <c r="J49" s="180"/>
-      <c r="K49" s="180"/>
-      <c r="L49" s="181"/>
-      <c r="M49" s="182" t="s">
+      <c r="G49" s="147"/>
+      <c r="H49" s="147"/>
+      <c r="I49" s="147"/>
+      <c r="J49" s="147"/>
+      <c r="K49" s="147"/>
+      <c r="L49" s="160"/>
+      <c r="M49" s="149" t="s">
         <v>12</v>
       </c>
-      <c r="N49" s="183"/>
+      <c r="N49" s="153"/>
     </row>
     <row r="50" spans="2:14" s="69" customFormat="1" ht="13">
-      <c r="B50" s="184" t="s">
+      <c r="B50" s="166" t="s">
         <v>149</v>
       </c>
-      <c r="C50" s="185"/>
-      <c r="D50" s="185"/>
-      <c r="E50" s="185"/>
-      <c r="F50" s="185"/>
-      <c r="G50" s="185"/>
-      <c r="H50" s="185"/>
-      <c r="I50" s="185"/>
-      <c r="J50" s="185"/>
-      <c r="K50" s="185"/>
-      <c r="L50" s="185"/>
-      <c r="M50" s="185"/>
-      <c r="N50" s="186"/>
+      <c r="C50" s="167"/>
+      <c r="D50" s="167"/>
+      <c r="E50" s="167"/>
+      <c r="F50" s="167"/>
+      <c r="G50" s="167"/>
+      <c r="H50" s="167"/>
+      <c r="I50" s="167"/>
+      <c r="J50" s="167"/>
+      <c r="K50" s="167"/>
+      <c r="L50" s="167"/>
+      <c r="M50" s="167"/>
+      <c r="N50" s="168"/>
     </row>
     <row r="51" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B51" s="65" t="s">
@@ -4473,19 +3700,19 @@
         <v>129</v>
       </c>
       <c r="E51" s="67"/>
-      <c r="F51" s="187" t="s">
+      <c r="F51" s="161" t="s">
         <v>130</v>
       </c>
-      <c r="G51" s="188"/>
-      <c r="H51" s="188"/>
-      <c r="I51" s="188"/>
-      <c r="J51" s="188"/>
-      <c r="K51" s="188"/>
-      <c r="L51" s="189"/>
-      <c r="M51" s="190" t="s">
+      <c r="G51" s="162"/>
+      <c r="H51" s="162"/>
+      <c r="I51" s="162"/>
+      <c r="J51" s="162"/>
+      <c r="K51" s="162"/>
+      <c r="L51" s="163"/>
+      <c r="M51" s="164" t="s">
         <v>131</v>
       </c>
-      <c r="N51" s="191"/>
+      <c r="N51" s="165"/>
     </row>
     <row r="52" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B52" s="66"/>
@@ -4496,89 +3723,89 @@
       <c r="E52" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="F52" s="179" t="s">
+      <c r="F52" s="159" t="s">
         <v>151</v>
       </c>
-      <c r="G52" s="180"/>
-      <c r="H52" s="180"/>
-      <c r="I52" s="180"/>
-      <c r="J52" s="180"/>
-      <c r="K52" s="180"/>
-      <c r="L52" s="181"/>
-      <c r="M52" s="182"/>
-      <c r="N52" s="183"/>
+      <c r="G52" s="147"/>
+      <c r="H52" s="147"/>
+      <c r="I52" s="147"/>
+      <c r="J52" s="147"/>
+      <c r="K52" s="147"/>
+      <c r="L52" s="160"/>
+      <c r="M52" s="149"/>
+      <c r="N52" s="153"/>
     </row>
     <row r="53" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B53" s="66"/>
       <c r="C53" s="66"/>
       <c r="D53" s="66"/>
       <c r="E53" s="67"/>
-      <c r="F53" s="179" t="s">
+      <c r="F53" s="159" t="s">
         <v>152</v>
       </c>
-      <c r="G53" s="180"/>
-      <c r="H53" s="180"/>
-      <c r="I53" s="180"/>
-      <c r="J53" s="180"/>
-      <c r="K53" s="180"/>
-      <c r="L53" s="181"/>
-      <c r="M53" s="182" t="s">
+      <c r="G53" s="147"/>
+      <c r="H53" s="147"/>
+      <c r="I53" s="147"/>
+      <c r="J53" s="147"/>
+      <c r="K53" s="147"/>
+      <c r="L53" s="160"/>
+      <c r="M53" s="149" t="s">
         <v>153</v>
       </c>
-      <c r="N53" s="183"/>
+      <c r="N53" s="153"/>
     </row>
     <row r="54" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B54" s="66"/>
       <c r="C54" s="66"/>
       <c r="D54" s="66"/>
       <c r="E54" s="67"/>
-      <c r="F54" s="179" t="s">
+      <c r="F54" s="159" t="s">
         <v>154</v>
       </c>
-      <c r="G54" s="180"/>
-      <c r="H54" s="180"/>
-      <c r="I54" s="180"/>
-      <c r="J54" s="180"/>
-      <c r="K54" s="180"/>
-      <c r="L54" s="181"/>
-      <c r="M54" s="182"/>
-      <c r="N54" s="183"/>
+      <c r="G54" s="147"/>
+      <c r="H54" s="147"/>
+      <c r="I54" s="147"/>
+      <c r="J54" s="147"/>
+      <c r="K54" s="147"/>
+      <c r="L54" s="160"/>
+      <c r="M54" s="149"/>
+      <c r="N54" s="153"/>
     </row>
     <row r="55" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B55" s="66"/>
       <c r="C55" s="66"/>
       <c r="D55" s="66"/>
       <c r="E55" s="67"/>
-      <c r="F55" s="179" t="s">
+      <c r="F55" s="159" t="s">
         <v>155</v>
       </c>
-      <c r="G55" s="180"/>
-      <c r="H55" s="180"/>
-      <c r="I55" s="180"/>
-      <c r="J55" s="180"/>
-      <c r="K55" s="180"/>
-      <c r="L55" s="181"/>
-      <c r="M55" s="182" t="s">
+      <c r="G55" s="147"/>
+      <c r="H55" s="147"/>
+      <c r="I55" s="147"/>
+      <c r="J55" s="147"/>
+      <c r="K55" s="147"/>
+      <c r="L55" s="160"/>
+      <c r="M55" s="149" t="s">
         <v>156</v>
       </c>
-      <c r="N55" s="183"/>
+      <c r="N55" s="153"/>
     </row>
     <row r="56" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B56" s="66"/>
       <c r="C56" s="66"/>
       <c r="D56" s="66"/>
       <c r="E56" s="67"/>
-      <c r="F56" s="179" t="s">
+      <c r="F56" s="159" t="s">
         <v>157</v>
       </c>
-      <c r="G56" s="180"/>
-      <c r="H56" s="180"/>
-      <c r="I56" s="180"/>
-      <c r="J56" s="180"/>
-      <c r="K56" s="180"/>
-      <c r="L56" s="181"/>
-      <c r="M56" s="182"/>
-      <c r="N56" s="183"/>
+      <c r="G56" s="147"/>
+      <c r="H56" s="147"/>
+      <c r="I56" s="147"/>
+      <c r="J56" s="147"/>
+      <c r="K56" s="147"/>
+      <c r="L56" s="160"/>
+      <c r="M56" s="149"/>
+      <c r="N56" s="153"/>
     </row>
     <row r="57" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B57" s="70"/>
@@ -4589,17 +3816,17 @@
       <c r="E57" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="F57" s="194" t="s">
+      <c r="F57" s="150" t="s">
         <v>158</v>
       </c>
-      <c r="G57" s="195"/>
-      <c r="H57" s="195"/>
-      <c r="I57" s="195"/>
-      <c r="J57" s="195"/>
-      <c r="K57" s="195"/>
-      <c r="L57" s="196"/>
-      <c r="M57" s="182"/>
-      <c r="N57" s="183"/>
+      <c r="G57" s="151"/>
+      <c r="H57" s="151"/>
+      <c r="I57" s="151"/>
+      <c r="J57" s="151"/>
+      <c r="K57" s="151"/>
+      <c r="L57" s="152"/>
+      <c r="M57" s="149"/>
+      <c r="N57" s="153"/>
     </row>
     <row r="58" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B58" s="76"/>
@@ -4610,17 +3837,17 @@
       <c r="E58" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="F58" s="197" t="s">
+      <c r="F58" s="154" t="s">
         <v>159</v>
       </c>
-      <c r="G58" s="198"/>
-      <c r="H58" s="198"/>
-      <c r="I58" s="198"/>
-      <c r="J58" s="198"/>
-      <c r="K58" s="198"/>
-      <c r="L58" s="199"/>
-      <c r="M58" s="200"/>
-      <c r="N58" s="201"/>
+      <c r="G58" s="155"/>
+      <c r="H58" s="155"/>
+      <c r="I58" s="155"/>
+      <c r="J58" s="155"/>
+      <c r="K58" s="155"/>
+      <c r="L58" s="156"/>
+      <c r="M58" s="157"/>
+      <c r="N58" s="158"/>
     </row>
     <row r="59" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B59" s="71"/>
@@ -4637,24 +3864,24 @@
       <c r="M59" s="78"/>
       <c r="N59" s="78"/>
     </row>
-    <row r="60" spans="2:14" s="69" customFormat="1" ht="14">
-      <c r="B60" s="202" t="s">
+    <row r="60" spans="2:14" s="69" customFormat="1" ht="15">
+      <c r="B60" s="144" t="s">
         <v>160</v>
       </c>
-      <c r="C60" s="202"/>
-      <c r="D60" s="202"/>
-      <c r="E60" s="202"/>
-      <c r="F60" s="202"/>
-      <c r="G60" s="202"/>
-      <c r="H60" s="202"/>
-      <c r="I60" s="202"/>
-      <c r="J60" s="202"/>
-      <c r="K60" s="202"/>
-      <c r="L60" s="202"/>
-      <c r="M60" s="202"/>
-      <c r="N60" s="202"/>
-    </row>
-    <row r="61" spans="2:14" s="69" customFormat="1" ht="14">
+      <c r="C60" s="144"/>
+      <c r="D60" s="144"/>
+      <c r="E60" s="144"/>
+      <c r="F60" s="144"/>
+      <c r="G60" s="144"/>
+      <c r="H60" s="144"/>
+      <c r="I60" s="144"/>
+      <c r="J60" s="144"/>
+      <c r="K60" s="144"/>
+      <c r="L60" s="144"/>
+      <c r="M60" s="144"/>
+      <c r="N60" s="144"/>
+    </row>
+    <row r="61" spans="2:14" s="69" customFormat="1" ht="15">
       <c r="B61" s="79"/>
       <c r="C61" s="79"/>
       <c r="D61" s="79"/>
@@ -4669,161 +3896,161 @@
       <c r="M61" s="79"/>
       <c r="N61" s="79"/>
     </row>
-    <row r="62" spans="2:14" s="69" customFormat="1" ht="14">
-      <c r="B62" s="203" t="s">
+    <row r="62" spans="2:14" s="69" customFormat="1" ht="15">
+      <c r="B62" s="145" t="s">
         <v>161</v>
       </c>
-      <c r="C62" s="144"/>
-      <c r="D62" s="144"/>
-      <c r="E62" s="144"/>
-      <c r="F62" s="144"/>
-      <c r="G62" s="144"/>
-      <c r="H62" s="144"/>
-      <c r="I62" s="144"/>
-      <c r="J62" s="144"/>
-      <c r="K62" s="144"/>
-      <c r="L62" s="144"/>
-      <c r="M62" s="144"/>
-      <c r="N62" s="144"/>
-    </row>
-    <row r="63" spans="2:14" s="69" customFormat="1" ht="27.5">
-      <c r="B63" s="192" t="s">
+      <c r="C62" s="143"/>
+      <c r="D62" s="143"/>
+      <c r="E62" s="143"/>
+      <c r="F62" s="143"/>
+      <c r="G62" s="143"/>
+      <c r="H62" s="143"/>
+      <c r="I62" s="143"/>
+      <c r="J62" s="143"/>
+      <c r="K62" s="143"/>
+      <c r="L62" s="143"/>
+      <c r="M62" s="143"/>
+      <c r="N62" s="143"/>
+    </row>
+    <row r="63" spans="2:14" s="69" customFormat="1" ht="28">
+      <c r="B63" s="146" t="s">
         <v>162</v>
       </c>
-      <c r="C63" s="192"/>
-      <c r="D63" s="192"/>
-      <c r="E63" s="192"/>
-      <c r="F63" s="192"/>
-      <c r="G63" s="192"/>
-      <c r="H63" s="192"/>
-      <c r="I63" s="192"/>
-      <c r="J63" s="192"/>
-      <c r="K63" s="192"/>
-      <c r="L63" s="192"/>
-      <c r="M63" s="192"/>
-      <c r="N63" s="192"/>
+      <c r="C63" s="146"/>
+      <c r="D63" s="146"/>
+      <c r="E63" s="146"/>
+      <c r="F63" s="146"/>
+      <c r="G63" s="146"/>
+      <c r="H63" s="146"/>
+      <c r="I63" s="146"/>
+      <c r="J63" s="146"/>
+      <c r="K63" s="146"/>
+      <c r="L63" s="146"/>
+      <c r="M63" s="146"/>
+      <c r="N63" s="146"/>
     </row>
     <row r="64" spans="2:14" s="69" customFormat="1" ht="13">
-      <c r="B64" s="182"/>
-      <c r="C64" s="193"/>
-      <c r="D64" s="193"/>
-      <c r="E64" s="193"/>
-      <c r="F64" s="193"/>
-      <c r="G64" s="193"/>
-      <c r="H64" s="193"/>
-      <c r="I64" s="193"/>
-      <c r="J64" s="193"/>
-      <c r="K64" s="193"/>
-      <c r="L64" s="193"/>
-      <c r="M64" s="193"/>
-      <c r="N64" s="193"/>
+      <c r="B64" s="149"/>
+      <c r="C64" s="148"/>
+      <c r="D64" s="148"/>
+      <c r="E64" s="148"/>
+      <c r="F64" s="148"/>
+      <c r="G64" s="148"/>
+      <c r="H64" s="148"/>
+      <c r="I64" s="148"/>
+      <c r="J64" s="148"/>
+      <c r="K64" s="148"/>
+      <c r="L64" s="148"/>
+      <c r="M64" s="148"/>
+      <c r="N64" s="148"/>
     </row>
     <row r="65" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B65" s="78"/>
       <c r="C65" s="78"/>
       <c r="D65" s="78"/>
       <c r="E65" s="80"/>
-      <c r="F65" s="180"/>
-      <c r="G65" s="180"/>
-      <c r="H65" s="180"/>
-      <c r="I65" s="180"/>
-      <c r="J65" s="180"/>
-      <c r="K65" s="180"/>
-      <c r="L65" s="180"/>
-      <c r="M65" s="193"/>
-      <c r="N65" s="193"/>
+      <c r="F65" s="147"/>
+      <c r="G65" s="147"/>
+      <c r="H65" s="147"/>
+      <c r="I65" s="147"/>
+      <c r="J65" s="147"/>
+      <c r="K65" s="147"/>
+      <c r="L65" s="147"/>
+      <c r="M65" s="148"/>
+      <c r="N65" s="148"/>
     </row>
     <row r="66" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B66" s="81"/>
       <c r="C66" s="78"/>
       <c r="D66" s="78"/>
       <c r="E66" s="80"/>
-      <c r="F66" s="180"/>
-      <c r="G66" s="180"/>
-      <c r="H66" s="180"/>
-      <c r="I66" s="180"/>
-      <c r="J66" s="180"/>
-      <c r="K66" s="180"/>
-      <c r="L66" s="180"/>
-      <c r="M66" s="193"/>
-      <c r="N66" s="193"/>
+      <c r="F66" s="147"/>
+      <c r="G66" s="147"/>
+      <c r="H66" s="147"/>
+      <c r="I66" s="147"/>
+      <c r="J66" s="147"/>
+      <c r="K66" s="147"/>
+      <c r="L66" s="147"/>
+      <c r="M66" s="148"/>
+      <c r="N66" s="148"/>
     </row>
     <row r="67" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B67" s="78"/>
       <c r="C67" s="78"/>
       <c r="D67" s="78"/>
       <c r="E67" s="80"/>
-      <c r="F67" s="180"/>
-      <c r="G67" s="180"/>
-      <c r="H67" s="180"/>
-      <c r="I67" s="180"/>
-      <c r="J67" s="180"/>
-      <c r="K67" s="180"/>
-      <c r="L67" s="180"/>
-      <c r="M67" s="193"/>
-      <c r="N67" s="193"/>
+      <c r="F67" s="147"/>
+      <c r="G67" s="147"/>
+      <c r="H67" s="147"/>
+      <c r="I67" s="147"/>
+      <c r="J67" s="147"/>
+      <c r="K67" s="147"/>
+      <c r="L67" s="147"/>
+      <c r="M67" s="148"/>
+      <c r="N67" s="148"/>
     </row>
     <row r="68" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B68" s="81"/>
       <c r="C68" s="78"/>
       <c r="D68" s="78"/>
       <c r="E68" s="78"/>
-      <c r="F68" s="180"/>
-      <c r="G68" s="180"/>
-      <c r="H68" s="180"/>
-      <c r="I68" s="180"/>
-      <c r="J68" s="180"/>
-      <c r="K68" s="180"/>
-      <c r="L68" s="180"/>
-      <c r="M68" s="193"/>
-      <c r="N68" s="193"/>
+      <c r="F68" s="147"/>
+      <c r="G68" s="147"/>
+      <c r="H68" s="147"/>
+      <c r="I68" s="147"/>
+      <c r="J68" s="147"/>
+      <c r="K68" s="147"/>
+      <c r="L68" s="147"/>
+      <c r="M68" s="148"/>
+      <c r="N68" s="148"/>
     </row>
     <row r="69" spans="2:14" s="69" customFormat="1" ht="13">
       <c r="B69" s="78"/>
       <c r="C69" s="78"/>
       <c r="D69" s="78"/>
       <c r="E69" s="78"/>
-      <c r="F69" s="180"/>
-      <c r="G69" s="180"/>
-      <c r="H69" s="180"/>
-      <c r="I69" s="180"/>
-      <c r="J69" s="180"/>
-      <c r="K69" s="180"/>
-      <c r="L69" s="180"/>
-      <c r="M69" s="193"/>
-      <c r="N69" s="193"/>
-    </row>
-    <row r="70" spans="2:14" ht="14">
-      <c r="B70" s="144"/>
-      <c r="C70" s="144"/>
-      <c r="D70" s="144"/>
-      <c r="E70" s="144"/>
-      <c r="F70" s="144"/>
-      <c r="G70" s="144"/>
-      <c r="H70" s="144"/>
-      <c r="I70" s="144"/>
-      <c r="J70" s="144"/>
-      <c r="K70" s="144"/>
-      <c r="L70" s="144"/>
-      <c r="M70" s="144"/>
-      <c r="N70" s="144"/>
-    </row>
-    <row r="71" spans="2:14" ht="14">
-      <c r="B71" s="202"/>
-      <c r="C71" s="202"/>
-      <c r="D71" s="202"/>
-      <c r="E71" s="202"/>
-      <c r="F71" s="202"/>
-      <c r="G71" s="202"/>
-      <c r="H71" s="202"/>
-      <c r="I71" s="202"/>
-      <c r="J71" s="202"/>
-      <c r="K71" s="202"/>
-      <c r="L71" s="202"/>
-      <c r="M71" s="202"/>
-      <c r="N71" s="202"/>
-    </row>
-    <row r="72" spans="2:14" ht="14">
+      <c r="F69" s="147"/>
+      <c r="G69" s="147"/>
+      <c r="H69" s="147"/>
+      <c r="I69" s="147"/>
+      <c r="J69" s="147"/>
+      <c r="K69" s="147"/>
+      <c r="L69" s="147"/>
+      <c r="M69" s="148"/>
+      <c r="N69" s="148"/>
+    </row>
+    <row r="70" spans="2:14" ht="15">
+      <c r="B70" s="143"/>
+      <c r="C70" s="143"/>
+      <c r="D70" s="143"/>
+      <c r="E70" s="143"/>
+      <c r="F70" s="143"/>
+      <c r="G70" s="143"/>
+      <c r="H70" s="143"/>
+      <c r="I70" s="143"/>
+      <c r="J70" s="143"/>
+      <c r="K70" s="143"/>
+      <c r="L70" s="143"/>
+      <c r="M70" s="143"/>
+      <c r="N70" s="143"/>
+    </row>
+    <row r="71" spans="2:14" ht="15">
+      <c r="B71" s="144"/>
+      <c r="C71" s="144"/>
+      <c r="D71" s="144"/>
+      <c r="E71" s="144"/>
+      <c r="F71" s="144"/>
+      <c r="G71" s="144"/>
+      <c r="H71" s="144"/>
+      <c r="I71" s="144"/>
+      <c r="J71" s="144"/>
+      <c r="K71" s="144"/>
+      <c r="L71" s="144"/>
+      <c r="M71" s="144"/>
+      <c r="N71" s="144"/>
+    </row>
+    <row r="72" spans="2:14" ht="15">
       <c r="B72" s="79"/>
       <c r="C72" s="79"/>
       <c r="D72" s="79"/>
@@ -4838,111 +4065,110 @@
       <c r="M72" s="79"/>
       <c r="N72" s="79"/>
     </row>
-    <row r="73" spans="2:14" ht="14">
-      <c r="B73" s="203"/>
-      <c r="C73" s="144"/>
-      <c r="D73" s="144"/>
-      <c r="E73" s="144"/>
-      <c r="F73" s="144"/>
-      <c r="G73" s="144"/>
-      <c r="H73" s="144"/>
-      <c r="I73" s="144"/>
-      <c r="J73" s="144"/>
-      <c r="K73" s="144"/>
-      <c r="L73" s="144"/>
-      <c r="M73" s="144"/>
-      <c r="N73" s="144"/>
-    </row>
-    <row r="74" spans="2:14" ht="27.5">
-      <c r="B74" s="192"/>
-      <c r="C74" s="192"/>
-      <c r="D74" s="192"/>
-      <c r="E74" s="192"/>
-      <c r="F74" s="192"/>
-      <c r="G74" s="192"/>
-      <c r="H74" s="192"/>
-      <c r="I74" s="192"/>
-      <c r="J74" s="192"/>
-      <c r="K74" s="192"/>
-      <c r="L74" s="192"/>
-      <c r="M74" s="192"/>
-      <c r="N74" s="192"/>
+    <row r="73" spans="2:14" ht="15">
+      <c r="B73" s="145"/>
+      <c r="C73" s="143"/>
+      <c r="D73" s="143"/>
+      <c r="E73" s="143"/>
+      <c r="F73" s="143"/>
+      <c r="G73" s="143"/>
+      <c r="H73" s="143"/>
+      <c r="I73" s="143"/>
+      <c r="J73" s="143"/>
+      <c r="K73" s="143"/>
+      <c r="L73" s="143"/>
+      <c r="M73" s="143"/>
+      <c r="N73" s="143"/>
+    </row>
+    <row r="74" spans="2:14" ht="28">
+      <c r="B74" s="146"/>
+      <c r="C74" s="146"/>
+      <c r="D74" s="146"/>
+      <c r="E74" s="146"/>
+      <c r="F74" s="146"/>
+      <c r="G74" s="146"/>
+      <c r="H74" s="146"/>
+      <c r="I74" s="146"/>
+      <c r="J74" s="146"/>
+      <c r="K74" s="146"/>
+      <c r="L74" s="146"/>
+      <c r="M74" s="146"/>
+      <c r="N74" s="146"/>
     </row>
   </sheetData>
   <mergeCells count="161">
-    <mergeCell ref="B70:N70"/>
-    <mergeCell ref="B71:N71"/>
-    <mergeCell ref="B73:N73"/>
-    <mergeCell ref="B74:N74"/>
-    <mergeCell ref="F67:L67"/>
-    <mergeCell ref="M67:N67"/>
-    <mergeCell ref="F68:L68"/>
-    <mergeCell ref="M68:N68"/>
-    <mergeCell ref="F69:L69"/>
-    <mergeCell ref="M69:N69"/>
-    <mergeCell ref="B63:N63"/>
-    <mergeCell ref="B64:N64"/>
-    <mergeCell ref="F65:L65"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="F66:L66"/>
-    <mergeCell ref="M66:N66"/>
-    <mergeCell ref="F57:L57"/>
-    <mergeCell ref="M57:N57"/>
-    <mergeCell ref="F58:L58"/>
-    <mergeCell ref="M58:N58"/>
-    <mergeCell ref="B60:N60"/>
-    <mergeCell ref="B62:N62"/>
-    <mergeCell ref="F54:L54"/>
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="F55:L55"/>
-    <mergeCell ref="M55:N55"/>
-    <mergeCell ref="F56:L56"/>
-    <mergeCell ref="M56:N56"/>
-    <mergeCell ref="F51:L51"/>
-    <mergeCell ref="M51:N51"/>
-    <mergeCell ref="F52:L52"/>
-    <mergeCell ref="M52:N52"/>
-    <mergeCell ref="F53:L53"/>
-    <mergeCell ref="M53:N53"/>
-    <mergeCell ref="F47:L47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="M48:N48"/>
-    <mergeCell ref="F49:L49"/>
-    <mergeCell ref="M49:N49"/>
-    <mergeCell ref="B50:N50"/>
-    <mergeCell ref="B43:N43"/>
-    <mergeCell ref="F44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="F45:L45"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="F46:L46"/>
-    <mergeCell ref="M46:N46"/>
-    <mergeCell ref="F39:L39"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="F40:L40"/>
-    <mergeCell ref="F41:L41"/>
-    <mergeCell ref="M41:N41"/>
-    <mergeCell ref="F42:L42"/>
-    <mergeCell ref="M42:N42"/>
-    <mergeCell ref="F36:L36"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="F37:L37"/>
-    <mergeCell ref="M37:N37"/>
-    <mergeCell ref="F38:L38"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="F32:L32"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="F33:L33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="F35:L35"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="F29:L29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="F30:L30"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="F31:L31"/>
-    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="E2:N2"/>
+    <mergeCell ref="B5:N5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:N7"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="B11:N11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:N8"/>
+    <mergeCell ref="B9:C10"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="B13:C14"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="H20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H21:L21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="D25:L25"/>
     <mergeCell ref="M25:N25"/>
@@ -4959,81 +4185,854 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="D24:L24"/>
     <mergeCell ref="M24:N24"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:L21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="B13:C14"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="B11:N11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:L12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:N8"/>
-    <mergeCell ref="B9:C10"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="E2:N2"/>
-    <mergeCell ref="B5:N5"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:N7"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="F32:L32"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="F33:L33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="B34:N34"/>
+    <mergeCell ref="F35:L35"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="F29:L29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="F30:L30"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="F31:L31"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="F39:L39"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="F40:L40"/>
+    <mergeCell ref="F41:L41"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="F42:L42"/>
+    <mergeCell ref="M42:N42"/>
+    <mergeCell ref="F36:L36"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="F37:L37"/>
+    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="F38:L38"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="F47:L47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="M48:N48"/>
+    <mergeCell ref="F49:L49"/>
+    <mergeCell ref="M49:N49"/>
+    <mergeCell ref="B50:N50"/>
+    <mergeCell ref="B43:N43"/>
+    <mergeCell ref="F44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="F45:L45"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="F46:L46"/>
+    <mergeCell ref="M46:N46"/>
+    <mergeCell ref="F54:L54"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="F55:L55"/>
+    <mergeCell ref="M55:N55"/>
+    <mergeCell ref="F56:L56"/>
+    <mergeCell ref="M56:N56"/>
+    <mergeCell ref="F51:L51"/>
+    <mergeCell ref="M51:N51"/>
+    <mergeCell ref="F52:L52"/>
+    <mergeCell ref="M52:N52"/>
+    <mergeCell ref="F53:L53"/>
+    <mergeCell ref="M53:N53"/>
+    <mergeCell ref="B63:N63"/>
+    <mergeCell ref="B64:N64"/>
+    <mergeCell ref="F65:L65"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="F66:L66"/>
+    <mergeCell ref="M66:N66"/>
+    <mergeCell ref="F57:L57"/>
+    <mergeCell ref="M57:N57"/>
+    <mergeCell ref="F58:L58"/>
+    <mergeCell ref="M58:N58"/>
+    <mergeCell ref="B60:N60"/>
+    <mergeCell ref="B62:N62"/>
+    <mergeCell ref="B70:N70"/>
+    <mergeCell ref="B71:N71"/>
+    <mergeCell ref="B73:N73"/>
+    <mergeCell ref="B74:N74"/>
+    <mergeCell ref="F67:L67"/>
+    <mergeCell ref="M67:N67"/>
+    <mergeCell ref="F68:L68"/>
+    <mergeCell ref="M68:N68"/>
+    <mergeCell ref="F69:L69"/>
+    <mergeCell ref="M69:N69"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="9" style="32"/>
+    <col min="2" max="2" width="8.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="33" style="32" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="32" customWidth="1"/>
+    <col min="6" max="6" width="10" style="32" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" style="32" customWidth="1"/>
+    <col min="8" max="8" width="25.1640625" style="32" customWidth="1"/>
+    <col min="9" max="11" width="8.6640625" style="32" customWidth="1"/>
+    <col min="12" max="13" width="9" style="32"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="16.5" customHeight="1" thickBot="1"/>
+    <row r="2" spans="1:13" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B2" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="91"/>
+      <c r="D2" s="84" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="92" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="94"/>
+    </row>
+    <row r="3" spans="1:13" ht="33.75" customHeight="1">
+      <c r="B3" s="95" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="96"/>
+      <c r="D3" s="57" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="97" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="99"/>
+    </row>
+    <row r="4" spans="1:13" ht="33.75" customHeight="1" thickBot="1">
+      <c r="B4" s="106" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="107"/>
+      <c r="D4" s="53" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="100"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="102"/>
+    </row>
+    <row r="5" spans="1:13" ht="33.75" customHeight="1">
+      <c r="B5" s="108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="109"/>
+      <c r="D5" s="9">
+        <v>8</v>
+      </c>
+      <c r="E5" s="100"/>
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="102"/>
+    </row>
+    <row r="6" spans="1:13" ht="22.5" customHeight="1">
+      <c r="B6" s="110" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="111"/>
+      <c r="D6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="100"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="102"/>
+    </row>
+    <row r="7" spans="1:13" ht="29.25" customHeight="1">
+      <c r="B7" s="110" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="111"/>
+      <c r="D7" s="56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="100"/>
+      <c r="F7" s="101"/>
+      <c r="G7" s="101"/>
+      <c r="H7" s="102"/>
+    </row>
+    <row r="8" spans="1:13" ht="27.75" customHeight="1">
+      <c r="B8" s="112" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="12">
+        <f>H37</f>
+        <v>983.5</v>
+      </c>
+      <c r="E8" s="100"/>
+      <c r="F8" s="101"/>
+      <c r="G8" s="101"/>
+      <c r="H8" s="102"/>
+    </row>
+    <row r="9" spans="1:13" ht="27" customHeight="1">
+      <c r="B9" s="113"/>
+      <c r="C9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="11">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="100"/>
+      <c r="F9" s="101"/>
+      <c r="G9" s="101"/>
+      <c r="H9" s="102"/>
+    </row>
+    <row r="10" spans="1:13" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B10" s="114"/>
+      <c r="C10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="13">
+        <f>D8*D9</f>
+        <v>983500</v>
+      </c>
+      <c r="E10" s="103"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="105"/>
+    </row>
+    <row r="11" spans="1:13" ht="38.25" customHeight="1" thickBot="1">
+      <c r="B11" s="115" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="115"/>
+      <c r="D11" s="82" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="120" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="121"/>
+      <c r="G11" s="121"/>
+      <c r="H11" s="121"/>
+    </row>
+    <row r="12" spans="1:13" ht="22.5" customHeight="1">
+      <c r="B12" s="116" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="118" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="118" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="118" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="118" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="118"/>
+      <c r="H12" s="122" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
+      <c r="A13" s="2"/>
+      <c r="B13" s="117"/>
+      <c r="C13" s="119"/>
+      <c r="D13" s="119"/>
+      <c r="E13" s="119"/>
+      <c r="F13" s="86" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="86" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="123"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="23.25" customHeight="1">
+      <c r="A14" s="2"/>
+      <c r="B14" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="14">
+        <v>220</v>
+      </c>
+      <c r="F14" s="14">
+        <v>3</v>
+      </c>
+      <c r="G14" s="14">
+        <v>4</v>
+      </c>
+      <c r="H14" s="15">
+        <f>E14*F14*G14</f>
+        <v>2640</v>
+      </c>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="21" customHeight="1" thickBot="1">
+      <c r="A15" s="2"/>
+      <c r="B15" s="133"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="17">
+        <v>0</v>
+      </c>
+      <c r="F15" s="17">
+        <v>0</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0</v>
+      </c>
+      <c r="H15" s="18">
+        <f>SUM(E15*F15*G15)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A16" s="2"/>
+      <c r="B16" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="88" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="20">
+        <v>500</v>
+      </c>
+      <c r="F16" s="21">
+        <v>4</v>
+      </c>
+      <c r="G16" s="21">
+        <v>1</v>
+      </c>
+      <c r="H16" s="15">
+        <f t="shared" ref="H16:H26" si="0">E16*F16*G16</f>
+        <v>2000</v>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+    </row>
+    <row r="17" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B17" s="125"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="35">
+        <v>60</v>
+      </c>
+      <c r="F17" s="36">
+        <v>1</v>
+      </c>
+      <c r="G17" s="36">
+        <v>1</v>
+      </c>
+      <c r="H17" s="33">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B18" s="125"/>
+      <c r="C18" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="24">
+        <v>0</v>
+      </c>
+      <c r="F18" s="37">
+        <v>0</v>
+      </c>
+      <c r="G18" s="37">
+        <v>0</v>
+      </c>
+      <c r="H18" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B19" s="126" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="85" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="46">
+        <v>1000</v>
+      </c>
+      <c r="F19" s="38">
+        <v>1</v>
+      </c>
+      <c r="G19" s="38">
+        <v>1</v>
+      </c>
+      <c r="H19" s="39">
+        <f t="shared" si="0"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B20" s="127"/>
+      <c r="C20" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="47">
+        <v>10</v>
+      </c>
+      <c r="F20" s="40">
+        <v>3</v>
+      </c>
+      <c r="G20" s="40">
+        <v>8</v>
+      </c>
+      <c r="H20" s="25">
+        <f t="shared" si="0"/>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B21" s="128" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="130" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="48">
+        <v>20</v>
+      </c>
+      <c r="F21" s="36">
+        <v>1</v>
+      </c>
+      <c r="G21" s="36">
+        <v>8</v>
+      </c>
+      <c r="H21" s="39">
+        <f t="shared" si="0"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B22" s="129"/>
+      <c r="C22" s="131"/>
+      <c r="D22" s="34" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="49">
+        <v>31</v>
+      </c>
+      <c r="F22" s="36">
+        <v>1</v>
+      </c>
+      <c r="G22" s="36">
+        <v>8</v>
+      </c>
+      <c r="H22" s="33">
+        <f t="shared" si="0"/>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B23" s="129"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="49">
+        <v>20</v>
+      </c>
+      <c r="F23" s="36">
+        <v>1</v>
+      </c>
+      <c r="G23" s="36">
+        <v>8</v>
+      </c>
+      <c r="H23" s="33">
+        <f t="shared" si="0"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B24" s="129"/>
+      <c r="C24" s="131"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="54">
+        <v>0</v>
+      </c>
+      <c r="F24" s="37">
+        <v>1</v>
+      </c>
+      <c r="G24" s="37">
+        <v>0</v>
+      </c>
+      <c r="H24" s="44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="22.5" customHeight="1">
+      <c r="B25" s="129"/>
+      <c r="C25" s="131"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="54">
+        <v>0</v>
+      </c>
+      <c r="F25" s="37">
+        <v>1</v>
+      </c>
+      <c r="G25" s="37">
+        <v>0</v>
+      </c>
+      <c r="H25" s="44">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B26" s="129"/>
+      <c r="C26" s="131"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="54">
+        <v>0</v>
+      </c>
+      <c r="F26" s="37">
+        <v>1</v>
+      </c>
+      <c r="G26" s="37">
+        <v>0</v>
+      </c>
+      <c r="H26" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B27" s="136" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="137" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="55">
+        <v>20</v>
+      </c>
+      <c r="F27" s="38">
+        <v>1</v>
+      </c>
+      <c r="G27" s="38">
+        <v>8</v>
+      </c>
+      <c r="H27" s="39">
+        <f>E27*F27*G27</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B28" s="124"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="E28" s="50">
+        <v>32</v>
+      </c>
+      <c r="F28" s="36">
+        <v>1</v>
+      </c>
+      <c r="G28" s="36">
+        <v>8</v>
+      </c>
+      <c r="H28" s="44">
+        <f t="shared" ref="H28:H35" si="1">E28*F28*G28</f>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B29" s="124"/>
+      <c r="C29" s="131"/>
+      <c r="D29" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="E29" s="50">
+        <v>18</v>
+      </c>
+      <c r="F29" s="36">
+        <v>1</v>
+      </c>
+      <c r="G29" s="36">
+        <v>8</v>
+      </c>
+      <c r="H29" s="44">
+        <f t="shared" si="1"/>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B30" s="124"/>
+      <c r="C30" s="131"/>
+      <c r="D30" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="50">
+        <v>20</v>
+      </c>
+      <c r="F30" s="36">
+        <v>1</v>
+      </c>
+      <c r="G30" s="36">
+        <v>8</v>
+      </c>
+      <c r="H30" s="44">
+        <f t="shared" si="1"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B31" s="124"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="50">
+        <v>55</v>
+      </c>
+      <c r="F31" s="36">
+        <v>1</v>
+      </c>
+      <c r="G31" s="36">
+        <v>8</v>
+      </c>
+      <c r="H31" s="44">
+        <f t="shared" si="1"/>
+        <v>440</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B32" s="124"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="E32" s="50">
+        <v>25</v>
+      </c>
+      <c r="F32" s="36">
+        <v>1</v>
+      </c>
+      <c r="G32" s="36">
+        <v>8</v>
+      </c>
+      <c r="H32" s="44">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B33" s="124"/>
+      <c r="C33" s="131"/>
+      <c r="D33" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="50">
+        <v>0</v>
+      </c>
+      <c r="F33" s="36">
+        <v>1</v>
+      </c>
+      <c r="G33" s="36">
+        <v>0</v>
+      </c>
+      <c r="H33" s="44">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B34" s="125"/>
+      <c r="C34" s="137" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" s="52">
+        <v>5</v>
+      </c>
+      <c r="F34" s="38">
+        <v>1</v>
+      </c>
+      <c r="G34" s="38">
+        <v>0</v>
+      </c>
+      <c r="H34" s="39">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B35" s="127"/>
+      <c r="C35" s="138"/>
+      <c r="D35" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="E35" s="51">
+        <v>5</v>
+      </c>
+      <c r="F35" s="40">
+        <v>1</v>
+      </c>
+      <c r="G35" s="40">
+        <v>0</v>
+      </c>
+      <c r="H35" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B36" s="139" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="140"/>
+      <c r="D36" s="140"/>
+      <c r="E36" s="140"/>
+      <c r="F36" s="140"/>
+      <c r="G36" s="140"/>
+      <c r="H36" s="6">
+        <f>SUM(H12:H35)</f>
+        <v>7868</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B37" s="141" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" s="142"/>
+      <c r="D37" s="142"/>
+      <c r="E37" s="142"/>
+      <c r="F37" s="142"/>
+      <c r="G37" s="142"/>
+      <c r="H37" s="4">
+        <f>H36/D5</f>
+        <v>983.5</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1">
+      <c r="B38" s="141" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="142"/>
+      <c r="D38" s="142"/>
+      <c r="E38" s="142"/>
+      <c r="F38" s="142"/>
+      <c r="G38" s="142"/>
+      <c r="H38" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B39" s="134" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="135"/>
+      <c r="D39" s="135"/>
+      <c r="E39" s="135"/>
+      <c r="F39" s="135"/>
+      <c r="G39" s="135"/>
+      <c r="H39" s="5">
+        <f>H37+H38</f>
+        <v>983.5</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" s="32" customFormat="1" ht="22.5" customHeight="1"/>
+    <row r="41" spans="2:8" s="32" customFormat="1" ht="16.5" customHeight="1"/>
+    <row r="42" spans="2:8" s="32" customFormat="1" ht="16.5" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B27:B35"/>
+    <mergeCell ref="C27:C33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B26"/>
+    <mergeCell ref="C21:C26"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:H10"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:B10"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>